<commit_message>
feat: add historical market data and configurations for stock risk monitoring
</commit_message>
<xml_diff>
--- a/outputs/monitor_xlsx/20260305.xlsx
+++ b/outputs/monitor_xlsx/20260305.xlsx
@@ -1087,7 +1087,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V17"/>
+  <dimension ref="A1:V20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2041,6 +2041,156 @@
         <v>8.960000000000001</v>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2454</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>聯發科</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>上市</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>1775</v>
+      </c>
+      <c r="E18" s="6" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="F18" t="n">
+        <v>8337</v>
+      </c>
+      <c r="G18" s="6" t="n">
+        <v>-1556</v>
+      </c>
+      <c r="H18" t="n">
+        <v>-9024</v>
+      </c>
+      <c r="I18" t="n">
+        <v>-9</v>
+      </c>
+      <c r="J18" t="n">
+        <v>512</v>
+      </c>
+      <c r="K18" t="n">
+        <v>500</v>
+      </c>
+      <c r="L18" t="n">
+        <v>5849</v>
+      </c>
+      <c r="M18" t="n">
+        <v>23256</v>
+      </c>
+      <c r="N18" t="n">
+        <v>-400923</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>3037</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>欣興</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>上市</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>450</v>
+      </c>
+      <c r="E19" s="6" t="n">
+        <v>7.91</v>
+      </c>
+      <c r="F19" t="n">
+        <v>18583</v>
+      </c>
+      <c r="G19" s="7" t="n">
+        <v>1513</v>
+      </c>
+      <c r="H19" t="n">
+        <v>-2702</v>
+      </c>
+      <c r="I19" t="n">
+        <v>708</v>
+      </c>
+      <c r="J19" t="n">
+        <v>-452</v>
+      </c>
+      <c r="K19" t="n">
+        <v>1840</v>
+      </c>
+      <c r="L19" t="n">
+        <v>39258</v>
+      </c>
+      <c r="M19" t="n">
+        <v>164587</v>
+      </c>
+      <c r="N19" t="n">
+        <v>-391991</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>8046</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>南電</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>上市</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>461</v>
+      </c>
+      <c r="E20" s="6" t="n">
+        <v>2.44</v>
+      </c>
+      <c r="F20" t="n">
+        <v>4226</v>
+      </c>
+      <c r="G20" s="7" t="n">
+        <v>28</v>
+      </c>
+      <c r="H20" t="n">
+        <v>2346</v>
+      </c>
+      <c r="I20" t="n">
+        <v>608</v>
+      </c>
+      <c r="J20" t="n">
+        <v>631</v>
+      </c>
+      <c r="K20" t="n">
+        <v>308</v>
+      </c>
+      <c r="L20" t="n">
+        <v>10048</v>
+      </c>
+      <c r="M20" t="n">
+        <v>44964</v>
+      </c>
+      <c r="N20" t="n">
+        <v>-161246</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:O1"/>

</xml_diff>